<commit_message>
unit and hmi codes
</commit_message>
<xml_diff>
--- a/vars_parsing.xlsx
+++ b/vars_parsing.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\d.sharygin\Desktop\Protocols\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F4D7E04-7372-42BA-90AB-7B2042BF228D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{852CA4D3-4ABC-4340-A224-2F05AE4BEEC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19095" yWindow="0" windowWidth="19410" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$I$52</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$B$1:$N$52</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="531" uniqueCount="352">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="653" uniqueCount="390">
   <si>
     <t>ЮТКБ.656463.300-001 РЭ</t>
   </si>
@@ -1098,6 +1098,120 @@
   </si>
   <si>
     <t>code_shet</t>
+  </si>
+  <si>
+    <t>code_order</t>
+  </si>
+  <si>
+    <t>ЮНИТ-М514-ВЧ-Р102-К103-К103-В101-В101-В120-М179.0700-В101-С01.03</t>
+  </si>
+  <si>
+    <t>ЮНИТ-М510-ВЧ-Р102-К101-В120-М179.0700-В101-С01.03</t>
+  </si>
+  <si>
+    <t>ЮНИТ-М510-ДЗЛ-Р102-К103-В101-В101-М179.0700-С04.03</t>
+  </si>
+  <si>
+    <t>ЮНИТ-М510-ДЗЛ-Р102-К101-х-В101-М179.0700-С04.03</t>
+  </si>
+  <si>
+    <t>ЮНИТ-М514-ЛВ-Р102-К103-К103-К103-В101-В101-В101-М179.0700-С01.03</t>
+  </si>
+  <si>
+    <t>ЮНИТ-М510-ЛВ-Р102-К101-х-В101-М179.0700-С01.03</t>
+  </si>
+  <si>
+    <t>ЮНИТ-М519-ДЗШ-Р102-К103-К103-К103-х-х-В101-В101-В101-В101-В101-М1С4.0С00-С01.03</t>
+  </si>
+  <si>
+    <t>ЮНИТ-М514-ДЗШ-Р102-К103-К103-х-х-В101-В101-М1С4.0С00-С01.03</t>
+  </si>
+  <si>
+    <t>ЮНИТ-М510-ДЗШ-Р102-К101-х-В101-М1С4.0С00-С01.03</t>
+  </si>
+  <si>
+    <t>ЮНИТ-М519-ДЗШ-Р102-К103-К103-К103-К103-К103-В121-В121-В101-М1С4.0С00-М1С4.0С00-С01.03</t>
+  </si>
+  <si>
+    <t>ЮНИТ-М519-ДЗШ-Р102-К103-К103-К103-В121-В121-В121-В121-В101-М1С4.0С00-М1С4.0С00-С01.03</t>
+  </si>
+  <si>
+    <t>ЮНИТ-М514-ДЗШ-Р102-К101-х-В101-В101-М1С4.0С00-М1С4.0С00-С01.03</t>
+  </si>
+  <si>
+    <t>ЮНИТ-М514-ДЗО-Р102-К103-К103-К103-х-В101-В101-М1С4.0С00-С01.03</t>
+  </si>
+  <si>
+    <t>ЮНИТ-М510-ДЗО-Р102-К101-х-В101-М1С4.0С00-С01.03</t>
+  </si>
+  <si>
+    <t>ЮНИТ-М514-ДЗО-Р102-К101-х-х-В101-М166.0600-М166.0600-С01.03</t>
+  </si>
+  <si>
+    <t>ЮНИТ-М519-ДЗТ-Р102-К103-К103-К103-В101-В101-В101-В101-В121-М186.0800-М186.0800-С01.03</t>
+  </si>
+  <si>
+    <t>ЮНИТ-М514-ДЗТ-Р102-К101-х-х-В101-М186.0800-М186.0800-С01.03</t>
+  </si>
+  <si>
+    <t>ЮНИТ-М514-РЗТ-Р102-К103-К103-х-В101-В101-В101-М168.0600-С01.03</t>
+  </si>
+  <si>
+    <t>ЮНИТ-М510-РЗТ-Р102-К101-х-В101-М168.0600-С01.03</t>
+  </si>
+  <si>
+    <t>ЮНИТ-М519-РЗТ-Р102-К103-К103-К103-К103-К103-К103-К103-В101-В101-В101-М168.0600-С01.03</t>
+  </si>
+  <si>
+    <t>ЮНИТ-М514-СВ-Р102-К103-К103-х-В101-В101-В101-М139.0300-С01.03</t>
+  </si>
+  <si>
+    <t>ЮНИТ-М510-СВ-Р102-К101-х-В101-М139.0300-С01.03</t>
+  </si>
+  <si>
+    <t>ЮНИТ-М514-БСК-Р102-К103-К103-В101-В101-М173.0700-М173.0700-С01.03</t>
+  </si>
+  <si>
+    <t>ЮНИТ-М514-БСК-Р102-К101-х-х-В101-М173.0700-М173.0700-С01.03</t>
+  </si>
+  <si>
+    <t>ЮНИТ-М514-БСК-Р102-К103-К103-х-В101-В101-В101-М141.0400-С01.03</t>
+  </si>
+  <si>
+    <t>code_order2</t>
+  </si>
+  <si>
+    <t>ЮНИТ-М519-ШР-Р102-К103-К103-К103-х-х-В101-В101-В101-В101-В101-М141.0400-С01.03</t>
+  </si>
+  <si>
+    <t>ЮНИТ-М519-ШР-Р102-К103-К103-К103-В101-В101-В101-В101-В101-М186.0800-М186.0800-С01.03</t>
+  </si>
+  <si>
+    <t>ЮНИТ-М514-ШР-Р102-К101-х-х-В101-М186.0800-М186.0800-С01.03</t>
+  </si>
+  <si>
+    <t>ЮНИТ-М514-ШР-Р102-К103-К103-В101-В101-М186.0800-М186.0800-С01.03</t>
+  </si>
+  <si>
+    <t>code_hmi</t>
+  </si>
+  <si>
+    <t>ЮНИТ-ИЧМ-КУГР</t>
+  </si>
+  <si>
+    <t>ЮНИТ-ИЧМ-СУГР-К-С</t>
+  </si>
+  <si>
+    <t>ЮНИТ-ИЧМ-СУГР-С</t>
+  </si>
+  <si>
+    <t>code_hmi2</t>
+  </si>
+  <si>
+    <t>ЮНИТ-ИЧМ-МНГР-К-К-С</t>
+  </si>
+  <si>
+    <t>ЮНИТ-ИЧМ-СУГР-К</t>
   </si>
 </sst>
 </file>
@@ -1149,7 +1263,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -1196,11 +1310,33 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1243,6 +1379,21 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1524,15 +1675,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M52"/>
+  <dimension ref="A1:Q52"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="121.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="121.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="7.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.140625" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="26.7109375" customWidth="1"/>
     <col min="8" max="8" width="24.85546875" customWidth="1"/>
     <col min="9" max="9" width="24.28515625" customWidth="1"/>
@@ -1540,26 +1691,30 @@
     <col min="11" max="11" width="25.28515625" customWidth="1"/>
     <col min="12" max="12" width="20.5703125" customWidth="1"/>
     <col min="13" max="13" width="23" customWidth="1"/>
+    <col min="14" max="14" width="89.42578125" customWidth="1"/>
+    <col min="15" max="15" width="86.140625" customWidth="1"/>
+    <col min="16" max="16" width="26.85546875" customWidth="1"/>
+    <col min="17" max="17" width="23.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
+        <v>158</v>
+      </c>
+      <c r="B1" s="6" t="s">
         <v>101</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="C1" s="6" t="s">
         <v>102</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="D1" s="6" t="s">
         <v>154</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="E1" s="6" t="s">
         <v>155</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="F1" s="6" t="s">
         <v>156</v>
-      </c>
-      <c r="F1" s="6" t="s">
-        <v>158</v>
       </c>
       <c r="G1" s="7" t="s">
         <v>306</v>
@@ -1582,25 +1737,37 @@
       <c r="M1" s="8" t="s">
         <v>351</v>
       </c>
-    </row>
-    <row r="2" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+      <c r="N1" s="8" t="s">
+        <v>352</v>
+      </c>
+      <c r="O1" s="17" t="s">
+        <v>378</v>
+      </c>
+      <c r="P1" s="21" t="s">
+        <v>383</v>
+      </c>
+      <c r="Q1" s="21" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="10" t="s">
+        <v>159</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>211</v>
       </c>
-      <c r="B2" s="9" t="s">
+      <c r="C2" s="9" t="s">
         <v>255</v>
       </c>
-      <c r="C2" s="10" t="s">
+      <c r="D2" s="10" t="s">
         <v>103</v>
       </c>
-      <c r="D2" s="10" t="s">
-        <v>157</v>
-      </c>
-      <c r="E2" s="11">
-        <v>46296</v>
-      </c>
-      <c r="F2" s="10" t="s">
-        <v>159</v>
+      <c r="E2" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="F2" s="11">
+        <v>46296</v>
       </c>
       <c r="G2" s="12" t="s">
         <v>310</v>
@@ -1619,25 +1786,33 @@
       <c r="M2" s="4" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
+      <c r="N2" s="16" t="s">
+        <v>359</v>
+      </c>
+      <c r="O2" s="19"/>
+      <c r="P2" s="18" t="s">
+        <v>384</v>
+      </c>
+      <c r="Q2" s="18"/>
+    </row>
+    <row r="3" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="10" t="s">
+        <v>160</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>212</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="C3" s="2" t="s">
         <v>256</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="D3" s="10" t="s">
         <v>104</v>
       </c>
-      <c r="D3" s="10" t="s">
-        <v>157</v>
-      </c>
-      <c r="E3" s="11">
-        <v>46296</v>
-      </c>
-      <c r="F3" s="10" t="s">
-        <v>160</v>
+      <c r="E3" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="F3" s="11">
+        <v>46296</v>
       </c>
       <c r="G3" s="12" t="s">
         <v>310</v>
@@ -1656,25 +1831,33 @@
       <c r="M3" s="3" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="4" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
+      <c r="N3" s="16" t="s">
+        <v>362</v>
+      </c>
+      <c r="O3" s="19"/>
+      <c r="P3" s="18" t="s">
+        <v>384</v>
+      </c>
+      <c r="Q3" s="18"/>
+    </row>
+    <row r="4" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="10" t="s">
+        <v>161</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>213</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="C4" s="2" t="s">
         <v>257</v>
       </c>
-      <c r="C4" s="10" t="s">
+      <c r="D4" s="10" t="s">
         <v>105</v>
       </c>
-      <c r="D4" s="10" t="s">
-        <v>157</v>
-      </c>
-      <c r="E4" s="11">
-        <v>46296</v>
-      </c>
-      <c r="F4" s="10" t="s">
-        <v>161</v>
+      <c r="E4" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="F4" s="11">
+        <v>46296</v>
       </c>
       <c r="G4" s="12" t="s">
         <v>310</v>
@@ -1693,25 +1876,33 @@
       <c r="M4" s="3" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="5" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
+      <c r="N4" s="16" t="s">
+        <v>359</v>
+      </c>
+      <c r="O4" s="19"/>
+      <c r="P4" s="18" t="s">
+        <v>384</v>
+      </c>
+      <c r="Q4" s="18"/>
+    </row>
+    <row r="5" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="10" t="s">
+        <v>162</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>214</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="C5" s="2" t="s">
         <v>258</v>
       </c>
-      <c r="C5" s="10" t="s">
+      <c r="D5" s="10" t="s">
         <v>106</v>
       </c>
-      <c r="D5" s="10" t="s">
-        <v>157</v>
-      </c>
-      <c r="E5" s="11">
-        <v>46296</v>
-      </c>
-      <c r="F5" s="10" t="s">
-        <v>162</v>
+      <c r="E5" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="F5" s="11">
+        <v>46296</v>
       </c>
       <c r="G5" s="12" t="s">
         <v>310</v>
@@ -1730,25 +1921,33 @@
       <c r="M5" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="6" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
+      <c r="N5" s="16" t="s">
+        <v>363</v>
+      </c>
+      <c r="O5" s="19"/>
+      <c r="P5" s="18" t="s">
+        <v>384</v>
+      </c>
+      <c r="Q5" s="18"/>
+    </row>
+    <row r="6" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="10" t="s">
+        <v>163</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>215</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="C6" s="2" t="s">
         <v>259</v>
       </c>
-      <c r="C6" s="10" t="s">
+      <c r="D6" s="10" t="s">
         <v>107</v>
       </c>
-      <c r="D6" s="10" t="s">
-        <v>157</v>
-      </c>
-      <c r="E6" s="11">
-        <v>46296</v>
-      </c>
-      <c r="F6" s="10" t="s">
-        <v>163</v>
+      <c r="E6" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="F6" s="11">
+        <v>46296</v>
       </c>
       <c r="G6" s="12" t="s">
         <v>307</v>
@@ -1767,25 +1966,37 @@
       <c r="M6" s="3" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="7" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
+      <c r="N6" s="15" t="s">
+        <v>365</v>
+      </c>
+      <c r="O6" s="19" t="s">
+        <v>365</v>
+      </c>
+      <c r="P6" s="18" t="s">
+        <v>384</v>
+      </c>
+      <c r="Q6" s="18" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="10" t="s">
+        <v>164</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>216</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="C7" s="2" t="s">
         <v>260</v>
       </c>
-      <c r="C7" s="10" t="s">
+      <c r="D7" s="10" t="s">
         <v>108</v>
       </c>
-      <c r="D7" s="10" t="s">
-        <v>157</v>
-      </c>
-      <c r="E7" s="11">
-        <v>46296</v>
-      </c>
-      <c r="F7" s="10" t="s">
-        <v>164</v>
+      <c r="E7" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="F7" s="11">
+        <v>46296</v>
       </c>
       <c r="G7" s="12" t="s">
         <v>308</v>
@@ -1804,25 +2015,33 @@
       <c r="M7" s="3" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="8" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
+      <c r="N7" s="15" t="s">
+        <v>365</v>
+      </c>
+      <c r="O7" s="19"/>
+      <c r="P7" s="18" t="s">
+        <v>384</v>
+      </c>
+      <c r="Q7" s="18"/>
+    </row>
+    <row r="8" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="10" t="s">
+        <v>165</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>217</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="C8" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="C8" s="10" t="s">
+      <c r="D8" s="10" t="s">
         <v>109</v>
       </c>
-      <c r="D8" s="10" t="s">
-        <v>157</v>
-      </c>
-      <c r="E8" s="11">
-        <v>46296</v>
-      </c>
-      <c r="F8" s="10" t="s">
-        <v>165</v>
+      <c r="E8" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="F8" s="11">
+        <v>46296</v>
       </c>
       <c r="G8" s="12" t="s">
         <v>308</v>
@@ -1841,25 +2060,33 @@
       <c r="M8" s="3" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="9" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="2" t="s">
+      <c r="N8" s="15" t="s">
+        <v>357</v>
+      </c>
+      <c r="O8" s="19"/>
+      <c r="P8" s="18" t="s">
+        <v>384</v>
+      </c>
+      <c r="Q8" s="18"/>
+    </row>
+    <row r="9" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="10" t="s">
+        <v>166</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>236</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="C9" s="2" t="s">
         <v>262</v>
       </c>
-      <c r="C9" s="10" t="s">
+      <c r="D9" s="10" t="s">
         <v>110</v>
       </c>
-      <c r="D9" s="10" t="s">
-        <v>157</v>
-      </c>
-      <c r="E9" s="11">
-        <v>46296</v>
-      </c>
-      <c r="F9" s="10" t="s">
-        <v>166</v>
+      <c r="E9" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="F9" s="11">
+        <v>46296</v>
       </c>
       <c r="G9" s="12" t="s">
         <v>308</v>
@@ -1878,25 +2105,33 @@
       <c r="M9" s="3" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="10" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
+      <c r="N9" s="16" t="s">
+        <v>373</v>
+      </c>
+      <c r="O9" s="19"/>
+      <c r="P9" s="18" t="s">
+        <v>384</v>
+      </c>
+      <c r="Q9" s="18"/>
+    </row>
+    <row r="10" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="10" t="s">
+        <v>167</v>
+      </c>
+      <c r="B10" s="2" t="s">
         <v>218</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="C10" s="2" t="s">
         <v>263</v>
       </c>
-      <c r="C10" s="10" t="s">
+      <c r="D10" s="10" t="s">
         <v>111</v>
       </c>
-      <c r="D10" s="10" t="s">
-        <v>157</v>
-      </c>
-      <c r="E10" s="11">
-        <v>46296</v>
-      </c>
-      <c r="F10" s="10" t="s">
-        <v>167</v>
+      <c r="E10" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="F10" s="11">
+        <v>46296</v>
       </c>
       <c r="G10" s="12" t="s">
         <v>308</v>
@@ -1915,25 +2150,33 @@
       <c r="M10" s="3" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="11" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="2" t="s">
+      <c r="N10" s="15" t="s">
+        <v>357</v>
+      </c>
+      <c r="O10" s="19"/>
+      <c r="P10" s="18" t="s">
+        <v>384</v>
+      </c>
+      <c r="Q10" s="18"/>
+    </row>
+    <row r="11" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="10" t="s">
+        <v>168</v>
+      </c>
+      <c r="B11" s="2" t="s">
         <v>210</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="C11" s="2" t="s">
         <v>264</v>
       </c>
-      <c r="C11" s="10" t="s">
+      <c r="D11" s="10" t="s">
         <v>112</v>
       </c>
-      <c r="D11" s="10" t="s">
-        <v>157</v>
-      </c>
-      <c r="E11" s="11">
-        <v>46296</v>
-      </c>
-      <c r="F11" s="10" t="s">
-        <v>168</v>
+      <c r="E11" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="F11" s="11">
+        <v>46296</v>
       </c>
       <c r="G11" s="12" t="s">
         <v>308</v>
@@ -1952,25 +2195,33 @@
       <c r="M11" s="3" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="12" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
+      <c r="N11" s="15" t="s">
+        <v>379</v>
+      </c>
+      <c r="O11" s="19"/>
+      <c r="P11" s="18" t="s">
+        <v>384</v>
+      </c>
+      <c r="Q11" s="18"/>
+    </row>
+    <row r="12" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="10" t="s">
+        <v>169</v>
+      </c>
+      <c r="B12" s="2" t="s">
         <v>237</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="C12" s="2" t="s">
         <v>265</v>
       </c>
-      <c r="C12" s="10" t="s">
+      <c r="D12" s="10" t="s">
         <v>113</v>
       </c>
-      <c r="D12" s="10" t="s">
-        <v>157</v>
-      </c>
-      <c r="E12" s="11">
-        <v>46296</v>
-      </c>
-      <c r="F12" s="10" t="s">
-        <v>169</v>
+      <c r="E12" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="F12" s="11">
+        <v>46296</v>
       </c>
       <c r="G12" s="12" t="s">
         <v>308</v>
@@ -1989,25 +2240,33 @@
       <c r="M12" s="3" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="13" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="2" t="s">
+      <c r="N12" s="16" t="s">
+        <v>353</v>
+      </c>
+      <c r="O12" s="19"/>
+      <c r="P12" s="18" t="s">
+        <v>384</v>
+      </c>
+      <c r="Q12" s="18"/>
+    </row>
+    <row r="13" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="10" t="s">
+        <v>170</v>
+      </c>
+      <c r="B13" s="2" t="s">
         <v>238</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="C13" s="2" t="s">
         <v>266</v>
       </c>
-      <c r="C13" s="10" t="s">
+      <c r="D13" s="10" t="s">
         <v>114</v>
       </c>
-      <c r="D13" s="10" t="s">
-        <v>157</v>
-      </c>
-      <c r="E13" s="11">
-        <v>46296</v>
-      </c>
-      <c r="F13" s="10" t="s">
-        <v>170</v>
+      <c r="E13" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="F13" s="11">
+        <v>46296</v>
       </c>
       <c r="G13" s="12" t="s">
         <v>308</v>
@@ -2026,25 +2285,33 @@
       <c r="M13" s="3" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="14" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="2" t="s">
+      <c r="N13" s="16" t="s">
+        <v>353</v>
+      </c>
+      <c r="O13" s="19"/>
+      <c r="P13" s="18" t="s">
+        <v>384</v>
+      </c>
+      <c r="Q13" s="18"/>
+    </row>
+    <row r="14" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="10" t="s">
+        <v>171</v>
+      </c>
+      <c r="B14" s="2" t="s">
         <v>239</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="C14" s="2" t="s">
         <v>267</v>
       </c>
-      <c r="C14" s="10" t="s">
+      <c r="D14" s="10" t="s">
         <v>115</v>
       </c>
-      <c r="D14" s="10" t="s">
-        <v>157</v>
-      </c>
-      <c r="E14" s="11">
-        <v>46296</v>
-      </c>
-      <c r="F14" s="10" t="s">
-        <v>171</v>
+      <c r="E14" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="F14" s="11">
+        <v>46296</v>
       </c>
       <c r="G14" s="12" t="s">
         <v>308</v>
@@ -2063,25 +2330,33 @@
       <c r="M14" s="3" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="15" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="2" t="s">
+      <c r="N14" s="16" t="s">
+        <v>353</v>
+      </c>
+      <c r="O14" s="19"/>
+      <c r="P14" s="18" t="s">
+        <v>384</v>
+      </c>
+      <c r="Q14" s="18"/>
+    </row>
+    <row r="15" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="B15" s="2" t="s">
         <v>240</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="C15" s="2" t="s">
         <v>268</v>
       </c>
-      <c r="C15" s="10" t="s">
+      <c r="D15" s="10" t="s">
         <v>116</v>
       </c>
-      <c r="D15" s="10" t="s">
-        <v>157</v>
-      </c>
-      <c r="E15" s="11">
-        <v>46296</v>
-      </c>
-      <c r="F15" s="10" t="s">
-        <v>172</v>
+      <c r="E15" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="F15" s="11">
+        <v>46296</v>
       </c>
       <c r="G15" s="12" t="s">
         <v>308</v>
@@ -2100,25 +2375,33 @@
       <c r="M15" s="3" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="16" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="2" t="s">
+      <c r="N15" s="16" t="s">
+        <v>353</v>
+      </c>
+      <c r="O15" s="19"/>
+      <c r="P15" s="18" t="s">
+        <v>384</v>
+      </c>
+      <c r="Q15" s="18"/>
+    </row>
+    <row r="16" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="10" t="s">
+        <v>173</v>
+      </c>
+      <c r="B16" s="2" t="s">
         <v>241</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="C16" s="2" t="s">
         <v>269</v>
       </c>
-      <c r="C16" s="10" t="s">
+      <c r="D16" s="10" t="s">
         <v>117</v>
       </c>
-      <c r="D16" s="10" t="s">
-        <v>157</v>
-      </c>
-      <c r="E16" s="11">
-        <v>46296</v>
-      </c>
-      <c r="F16" s="10" t="s">
-        <v>173</v>
+      <c r="E16" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="F16" s="11">
+        <v>46296</v>
       </c>
       <c r="G16" s="12" t="s">
         <v>308</v>
@@ -2137,25 +2420,33 @@
       <c r="M16" s="3" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="17" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="2" t="s">
+      <c r="N16" s="16" t="s">
+        <v>355</v>
+      </c>
+      <c r="O16" s="19"/>
+      <c r="P16" s="18" t="s">
+        <v>384</v>
+      </c>
+      <c r="Q16" s="18"/>
+    </row>
+    <row r="17" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="10" t="s">
+        <v>174</v>
+      </c>
+      <c r="B17" s="2" t="s">
         <v>242</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="C17" s="2" t="s">
         <v>270</v>
       </c>
-      <c r="C17" s="10" t="s">
+      <c r="D17" s="10" t="s">
         <v>118</v>
       </c>
-      <c r="D17" s="10" t="s">
-        <v>157</v>
-      </c>
-      <c r="E17" s="11">
-        <v>46296</v>
-      </c>
-      <c r="F17" s="10" t="s">
-        <v>174</v>
+      <c r="E17" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="F17" s="11">
+        <v>46296</v>
       </c>
       <c r="G17" s="12" t="s">
         <v>308</v>
@@ -2174,25 +2465,33 @@
       <c r="M17" s="3" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="18" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="2" t="s">
+      <c r="N17" s="16" t="s">
+        <v>355</v>
+      </c>
+      <c r="O17" s="19"/>
+      <c r="P17" s="18" t="s">
+        <v>384</v>
+      </c>
+      <c r="Q17" s="18"/>
+    </row>
+    <row r="18" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="10" t="s">
+        <v>175</v>
+      </c>
+      <c r="B18" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="C18" s="2" t="s">
         <v>271</v>
       </c>
-      <c r="C18" s="10" t="s">
+      <c r="D18" s="10" t="s">
         <v>119</v>
       </c>
-      <c r="D18" s="10" t="s">
-        <v>157</v>
-      </c>
-      <c r="E18" s="11">
-        <v>46296</v>
-      </c>
-      <c r="F18" s="10" t="s">
-        <v>175</v>
+      <c r="E18" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="F18" s="11">
+        <v>46296</v>
       </c>
       <c r="G18" s="12" t="s">
         <v>308</v>
@@ -2211,25 +2510,33 @@
       <c r="M18" s="3" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="19" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="2" t="s">
+      <c r="N18" s="15" t="s">
+        <v>357</v>
+      </c>
+      <c r="O18" s="19"/>
+      <c r="P18" s="18" t="s">
+        <v>384</v>
+      </c>
+      <c r="Q18" s="18"/>
+    </row>
+    <row r="19" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="10" t="s">
+        <v>176</v>
+      </c>
+      <c r="B19" s="2" t="s">
         <v>244</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="C19" s="2" t="s">
         <v>272</v>
       </c>
-      <c r="C19" s="10" t="s">
+      <c r="D19" s="10" t="s">
         <v>120</v>
       </c>
-      <c r="D19" s="10" t="s">
-        <v>157</v>
-      </c>
-      <c r="E19" s="11">
-        <v>46296</v>
-      </c>
-      <c r="F19" s="10" t="s">
-        <v>176</v>
+      <c r="E19" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="F19" s="11">
+        <v>46296</v>
       </c>
       <c r="G19" s="12" t="s">
         <v>308</v>
@@ -2248,25 +2555,33 @@
       <c r="M19" s="3" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="20" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="2" t="s">
+      <c r="N19" s="15" t="s">
+        <v>357</v>
+      </c>
+      <c r="O19" s="19"/>
+      <c r="P19" s="18" t="s">
+        <v>384</v>
+      </c>
+      <c r="Q19" s="18"/>
+    </row>
+    <row r="20" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="10" t="s">
+        <v>177</v>
+      </c>
+      <c r="B20" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="C20" s="2" t="s">
         <v>273</v>
       </c>
-      <c r="C20" s="10" t="s">
+      <c r="D20" s="10" t="s">
         <v>121</v>
       </c>
-      <c r="D20" s="10" t="s">
-        <v>157</v>
-      </c>
-      <c r="E20" s="11">
-        <v>46296</v>
-      </c>
-      <c r="F20" s="10" t="s">
-        <v>177</v>
+      <c r="E20" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="F20" s="11">
+        <v>46296</v>
       </c>
       <c r="G20" s="12" t="s">
         <v>308</v>
@@ -2285,25 +2600,33 @@
       <c r="M20" s="3" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="21" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="2" t="s">
+      <c r="N20" s="15" t="s">
+        <v>357</v>
+      </c>
+      <c r="O20" s="19"/>
+      <c r="P20" s="18" t="s">
+        <v>384</v>
+      </c>
+      <c r="Q20" s="18"/>
+    </row>
+    <row r="21" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="10" t="s">
+        <v>178</v>
+      </c>
+      <c r="B21" s="2" t="s">
         <v>220</v>
       </c>
-      <c r="B21" s="2" t="s">
+      <c r="C21" s="2" t="s">
         <v>274</v>
       </c>
-      <c r="C21" s="10" t="s">
+      <c r="D21" s="10" t="s">
         <v>122</v>
       </c>
-      <c r="D21" s="10" t="s">
-        <v>157</v>
-      </c>
-      <c r="E21" s="11">
-        <v>46296</v>
-      </c>
-      <c r="F21" s="10" t="s">
-        <v>178</v>
+      <c r="E21" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="F21" s="11">
+        <v>46296</v>
       </c>
       <c r="G21" s="12" t="s">
         <v>309</v>
@@ -2326,25 +2649,37 @@
       <c r="M21" s="3" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="22" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="2" t="s">
+      <c r="N21" s="16" t="s">
+        <v>368</v>
+      </c>
+      <c r="O21" s="20" t="s">
+        <v>365</v>
+      </c>
+      <c r="P21" s="18" t="s">
+        <v>386</v>
+      </c>
+      <c r="Q21" s="18" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="22" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="B22" s="2" t="s">
         <v>221</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="C22" s="2" t="s">
         <v>275</v>
       </c>
-      <c r="C22" s="10" t="s">
+      <c r="D22" s="10" t="s">
         <v>123</v>
       </c>
-      <c r="D22" s="10" t="s">
-        <v>157</v>
-      </c>
-      <c r="E22" s="11">
-        <v>46296</v>
-      </c>
-      <c r="F22" s="10" t="s">
-        <v>179</v>
+      <c r="E22" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="F22" s="11">
+        <v>46296</v>
       </c>
       <c r="G22" s="12" t="s">
         <v>308</v>
@@ -2363,25 +2698,33 @@
       <c r="M22" s="3" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="23" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="2" t="s">
+      <c r="N22" s="15" t="s">
+        <v>368</v>
+      </c>
+      <c r="O22" s="19"/>
+      <c r="P22" s="18" t="s">
+        <v>385</v>
+      </c>
+      <c r="Q22" s="18"/>
+    </row>
+    <row r="23" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="10" t="s">
+        <v>180</v>
+      </c>
+      <c r="B23" s="2" t="s">
         <v>222</v>
       </c>
-      <c r="B23" s="2" t="s">
+      <c r="C23" s="2" t="s">
         <v>276</v>
       </c>
-      <c r="C23" s="10" t="s">
+      <c r="D23" s="10" t="s">
         <v>124</v>
       </c>
-      <c r="D23" s="10" t="s">
-        <v>157</v>
-      </c>
-      <c r="E23" s="11">
-        <v>46296</v>
-      </c>
-      <c r="F23" s="10" t="s">
-        <v>180</v>
+      <c r="E23" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="F23" s="11">
+        <v>46296</v>
       </c>
       <c r="G23" s="12" t="s">
         <v>308</v>
@@ -2400,30 +2743,38 @@
       <c r="M23" s="3" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="24" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="2" t="s">
+      <c r="N23" s="16" t="s">
+        <v>370</v>
+      </c>
+      <c r="O23" s="19"/>
+      <c r="P23" s="18" t="s">
+        <v>384</v>
+      </c>
+      <c r="Q23" s="18"/>
+    </row>
+    <row r="24" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="10" t="s">
+        <v>181</v>
+      </c>
+      <c r="B24" s="2" t="s">
         <v>245</v>
       </c>
-      <c r="B24" s="2" t="s">
+      <c r="C24" s="2" t="s">
         <v>277</v>
       </c>
-      <c r="C24" s="10" t="s">
+      <c r="D24" s="10" t="s">
         <v>125</v>
       </c>
-      <c r="D24" s="10" t="s">
-        <v>157</v>
-      </c>
-      <c r="E24" s="11">
-        <v>46296</v>
-      </c>
-      <c r="F24" s="10" t="s">
-        <v>181</v>
+      <c r="E24" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="F24" s="11">
+        <v>46296</v>
       </c>
       <c r="G24" s="12" t="s">
         <v>309</v>
       </c>
-      <c r="H24" s="12" t="s">
+      <c r="H24" s="15" t="s">
         <v>322</v>
       </c>
       <c r="I24" s="13" t="s">
@@ -2441,25 +2792,37 @@
       <c r="M24" s="3" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="25" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="2" t="s">
+      <c r="N24" s="16" t="s">
+        <v>368</v>
+      </c>
+      <c r="O24" s="19" t="s">
+        <v>365</v>
+      </c>
+      <c r="P24" s="18" t="s">
+        <v>386</v>
+      </c>
+      <c r="Q24" s="18" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="25" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="10" t="s">
+        <v>182</v>
+      </c>
+      <c r="B25" s="2" t="s">
         <v>223</v>
       </c>
-      <c r="B25" s="2" t="s">
+      <c r="C25" s="2" t="s">
         <v>278</v>
       </c>
-      <c r="C25" s="10" t="s">
+      <c r="D25" s="10" t="s">
         <v>126</v>
       </c>
-      <c r="D25" s="10" t="s">
-        <v>157</v>
-      </c>
-      <c r="E25" s="11">
-        <v>46296</v>
-      </c>
-      <c r="F25" s="10" t="s">
-        <v>182</v>
+      <c r="E25" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="F25" s="11">
+        <v>46296</v>
       </c>
       <c r="G25" s="12" t="s">
         <v>308</v>
@@ -2478,25 +2841,33 @@
       <c r="M25" s="3" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="26" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="2" t="s">
+      <c r="N25" s="16" t="s">
+        <v>368</v>
+      </c>
+      <c r="O25" s="19"/>
+      <c r="P25" s="18" t="s">
+        <v>386</v>
+      </c>
+      <c r="Q25" s="18"/>
+    </row>
+    <row r="26" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="10" t="s">
+        <v>183</v>
+      </c>
+      <c r="B26" s="2" t="s">
         <v>224</v>
       </c>
-      <c r="B26" s="2" t="s">
+      <c r="C26" s="2" t="s">
         <v>279</v>
       </c>
-      <c r="C26" s="10" t="s">
+      <c r="D26" s="10" t="s">
         <v>127</v>
       </c>
-      <c r="D26" s="10" t="s">
-        <v>157</v>
-      </c>
-      <c r="E26" s="11">
-        <v>46296</v>
-      </c>
-      <c r="F26" s="10" t="s">
-        <v>183</v>
+      <c r="E26" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="F26" s="11">
+        <v>46296</v>
       </c>
       <c r="G26" s="12" t="s">
         <v>308</v>
@@ -2515,25 +2886,33 @@
       <c r="M26" s="3" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="27" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="2" t="s">
+      <c r="N26" s="15" t="s">
+        <v>372</v>
+      </c>
+      <c r="O26" s="19"/>
+      <c r="P26" s="18" t="s">
+        <v>384</v>
+      </c>
+      <c r="Q26" s="18"/>
+    </row>
+    <row r="27" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="10" t="s">
+        <v>184</v>
+      </c>
+      <c r="B27" s="2" t="s">
         <v>225</v>
       </c>
-      <c r="B27" s="2" t="s">
+      <c r="C27" s="2" t="s">
         <v>280</v>
       </c>
-      <c r="C27" s="10" t="s">
+      <c r="D27" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="D27" s="10" t="s">
-        <v>157</v>
-      </c>
-      <c r="E27" s="11">
-        <v>46296</v>
-      </c>
-      <c r="F27" s="10" t="s">
-        <v>184</v>
+      <c r="E27" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="F27" s="11">
+        <v>46296</v>
       </c>
       <c r="G27" s="12" t="s">
         <v>308</v>
@@ -2552,25 +2931,33 @@
       <c r="M27" s="3" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="28" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="2" t="s">
+      <c r="N27" s="16" t="s">
+        <v>375</v>
+      </c>
+      <c r="O27" s="19"/>
+      <c r="P27" s="18" t="s">
+        <v>384</v>
+      </c>
+      <c r="Q27" s="18"/>
+    </row>
+    <row r="28" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="10" t="s">
+        <v>185</v>
+      </c>
+      <c r="B28" s="2" t="s">
         <v>226</v>
       </c>
-      <c r="B28" s="2" t="s">
+      <c r="C28" s="2" t="s">
         <v>281</v>
       </c>
-      <c r="C28" s="10" t="s">
+      <c r="D28" s="10" t="s">
         <v>129</v>
       </c>
-      <c r="D28" s="10" t="s">
-        <v>157</v>
-      </c>
-      <c r="E28" s="11">
-        <v>46296</v>
-      </c>
-      <c r="F28" s="10" t="s">
-        <v>185</v>
+      <c r="E28" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="F28" s="11">
+        <v>46296</v>
       </c>
       <c r="G28" s="12" t="s">
         <v>309</v>
@@ -2589,25 +2976,37 @@
       <c r="M28" s="3" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="29" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="2" t="s">
+      <c r="N28" s="16" t="s">
+        <v>375</v>
+      </c>
+      <c r="O28" s="19" t="s">
+        <v>377</v>
+      </c>
+      <c r="P28" s="18" t="s">
+        <v>384</v>
+      </c>
+      <c r="Q28" s="18" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="29" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="10" t="s">
+        <v>186</v>
+      </c>
+      <c r="B29" s="2" t="s">
         <v>227</v>
       </c>
-      <c r="B29" s="2" t="s">
+      <c r="C29" s="2" t="s">
         <v>282</v>
       </c>
-      <c r="C29" s="10" t="s">
+      <c r="D29" s="10" t="s">
         <v>130</v>
       </c>
-      <c r="D29" s="10" t="s">
-        <v>157</v>
-      </c>
-      <c r="E29" s="11">
-        <v>46296</v>
-      </c>
-      <c r="F29" s="10" t="s">
-        <v>186</v>
+      <c r="E29" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="F29" s="11">
+        <v>46296</v>
       </c>
       <c r="G29" s="12" t="s">
         <v>308</v>
@@ -2626,25 +3025,33 @@
       <c r="M29" s="3" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="30" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="2" t="s">
+      <c r="N29" s="16" t="s">
+        <v>380</v>
+      </c>
+      <c r="O29" s="19"/>
+      <c r="P29" s="18" t="s">
+        <v>386</v>
+      </c>
+      <c r="Q29" s="18"/>
+    </row>
+    <row r="30" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="10" t="s">
+        <v>187</v>
+      </c>
+      <c r="B30" s="2" t="s">
         <v>228</v>
       </c>
-      <c r="B30" s="2" t="s">
+      <c r="C30" s="2" t="s">
         <v>283</v>
       </c>
-      <c r="C30" s="10" t="s">
+      <c r="D30" s="10" t="s">
         <v>131</v>
       </c>
-      <c r="D30" s="10" t="s">
-        <v>157</v>
-      </c>
-      <c r="E30" s="11">
-        <v>46296</v>
-      </c>
-      <c r="F30" s="10" t="s">
-        <v>187</v>
+      <c r="E30" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="F30" s="11">
+        <v>46296</v>
       </c>
       <c r="G30" s="12" t="s">
         <v>308</v>
@@ -2663,25 +3070,33 @@
       <c r="M30" s="3" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="31" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="2" t="s">
+      <c r="N30" s="16" t="s">
+        <v>380</v>
+      </c>
+      <c r="O30" s="19"/>
+      <c r="P30" s="18" t="s">
+        <v>384</v>
+      </c>
+      <c r="Q30" s="18"/>
+    </row>
+    <row r="31" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="10" t="s">
+        <v>188</v>
+      </c>
+      <c r="B31" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="B31" s="2" t="s">
+      <c r="C31" s="2" t="s">
         <v>284</v>
       </c>
-      <c r="C31" s="10" t="s">
+      <c r="D31" s="10" t="s">
         <v>132</v>
       </c>
-      <c r="D31" s="10" t="s">
-        <v>157</v>
-      </c>
-      <c r="E31" s="11">
-        <v>46296</v>
-      </c>
-      <c r="F31" s="10" t="s">
-        <v>188</v>
+      <c r="E31" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="F31" s="11">
+        <v>46296</v>
       </c>
       <c r="G31" s="12" t="s">
         <v>308</v>
@@ -2700,25 +3115,33 @@
       <c r="M31" s="3" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="32" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="2" t="s">
+      <c r="N31" s="16" t="s">
+        <v>382</v>
+      </c>
+      <c r="O31" s="19"/>
+      <c r="P31" s="18" t="s">
+        <v>384</v>
+      </c>
+      <c r="Q31" s="18"/>
+    </row>
+    <row r="32" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="10" t="s">
+        <v>189</v>
+      </c>
+      <c r="B32" s="2" t="s">
         <v>230</v>
       </c>
-      <c r="B32" s="2" t="s">
+      <c r="C32" s="2" t="s">
         <v>285</v>
       </c>
-      <c r="C32" s="10" t="s">
+      <c r="D32" s="10" t="s">
         <v>133</v>
       </c>
-      <c r="D32" s="10" t="s">
-        <v>157</v>
-      </c>
-      <c r="E32" s="11">
-        <v>46296</v>
-      </c>
-      <c r="F32" s="10" t="s">
-        <v>189</v>
+      <c r="E32" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="F32" s="11">
+        <v>46296</v>
       </c>
       <c r="G32" s="12" t="s">
         <v>308</v>
@@ -2737,25 +3160,33 @@
       <c r="M32" s="3" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="33" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="2" t="s">
+      <c r="N32" s="16" t="s">
+        <v>359</v>
+      </c>
+      <c r="O32" s="19"/>
+      <c r="P32" s="18" t="s">
+        <v>384</v>
+      </c>
+      <c r="Q32" s="18"/>
+    </row>
+    <row r="33" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="10" t="s">
+        <v>190</v>
+      </c>
+      <c r="B33" s="2" t="s">
         <v>246</v>
       </c>
-      <c r="B33" s="2" t="s">
+      <c r="C33" s="2" t="s">
         <v>286</v>
       </c>
-      <c r="C33" s="10" t="s">
+      <c r="D33" s="10" t="s">
         <v>134</v>
       </c>
-      <c r="D33" s="10" t="s">
-        <v>157</v>
-      </c>
-      <c r="E33" s="11">
-        <v>46296</v>
-      </c>
-      <c r="F33" s="10" t="s">
-        <v>190</v>
+      <c r="E33" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="F33" s="11">
+        <v>46296</v>
       </c>
       <c r="G33" s="12" t="s">
         <v>308</v>
@@ -2774,25 +3205,33 @@
       <c r="M33" s="3" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="34" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="2" t="s">
+      <c r="N33" s="16" t="s">
+        <v>361</v>
+      </c>
+      <c r="O33" s="19"/>
+      <c r="P33" s="18" t="s">
+        <v>385</v>
+      </c>
+      <c r="Q33" s="18"/>
+    </row>
+    <row r="34" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="10" t="s">
+        <v>191</v>
+      </c>
+      <c r="B34" s="2" t="s">
         <v>247</v>
       </c>
-      <c r="B34" s="2" t="s">
+      <c r="C34" s="2" t="s">
         <v>287</v>
       </c>
-      <c r="C34" s="10" t="s">
+      <c r="D34" s="10" t="s">
         <v>135</v>
       </c>
-      <c r="D34" s="10" t="s">
-        <v>157</v>
-      </c>
-      <c r="E34" s="11">
-        <v>46296</v>
-      </c>
-      <c r="F34" s="10" t="s">
-        <v>191</v>
+      <c r="E34" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="F34" s="11">
+        <v>46296</v>
       </c>
       <c r="G34" s="12" t="s">
         <v>308</v>
@@ -2811,25 +3250,33 @@
       <c r="M34" s="3" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="35" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="2" t="s">
+      <c r="N34" s="16" t="s">
+        <v>364</v>
+      </c>
+      <c r="O34" s="19"/>
+      <c r="P34" s="18" t="s">
+        <v>388</v>
+      </c>
+      <c r="Q34" s="18"/>
+    </row>
+    <row r="35" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="10" t="s">
+        <v>192</v>
+      </c>
+      <c r="B35" s="2" t="s">
         <v>248</v>
       </c>
-      <c r="B35" s="2" t="s">
+      <c r="C35" s="2" t="s">
         <v>288</v>
       </c>
-      <c r="C35" s="10" t="s">
+      <c r="D35" s="10" t="s">
         <v>136</v>
       </c>
-      <c r="D35" s="10" t="s">
-        <v>157</v>
-      </c>
-      <c r="E35" s="11">
-        <v>46296</v>
-      </c>
-      <c r="F35" s="10" t="s">
-        <v>192</v>
+      <c r="E35" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="F35" s="11">
+        <v>46296</v>
       </c>
       <c r="G35" s="12" t="s">
         <v>309</v>
@@ -2848,25 +3295,37 @@
       <c r="M35" s="3" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="36" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="2" t="s">
+      <c r="N35" s="15" t="s">
+        <v>367</v>
+      </c>
+      <c r="O35" s="19" t="s">
+        <v>367</v>
+      </c>
+      <c r="P35" s="18" t="s">
+        <v>385</v>
+      </c>
+      <c r="Q35" s="18" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="36" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="10" t="s">
+        <v>193</v>
+      </c>
+      <c r="B36" s="2" t="s">
         <v>231</v>
       </c>
-      <c r="B36" s="2" t="s">
+      <c r="C36" s="2" t="s">
         <v>289</v>
       </c>
-      <c r="C36" s="10" t="s">
+      <c r="D36" s="10" t="s">
         <v>137</v>
       </c>
-      <c r="D36" s="10" t="s">
-        <v>157</v>
-      </c>
-      <c r="E36" s="11">
-        <v>46296</v>
-      </c>
-      <c r="F36" s="10" t="s">
-        <v>193</v>
+      <c r="E36" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="F36" s="11">
+        <v>46296</v>
       </c>
       <c r="G36" s="12" t="s">
         <v>308</v>
@@ -2885,25 +3344,33 @@
       <c r="M36" s="3" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="37" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="2" t="s">
+      <c r="N36" s="15" t="s">
+        <v>367</v>
+      </c>
+      <c r="O36" s="19"/>
+      <c r="P36" s="18" t="s">
+        <v>385</v>
+      </c>
+      <c r="Q36" s="18"/>
+    </row>
+    <row r="37" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="10" t="s">
+        <v>194</v>
+      </c>
+      <c r="B37" s="2" t="s">
         <v>217</v>
       </c>
-      <c r="B37" s="2" t="s">
+      <c r="C37" s="2" t="s">
         <v>290</v>
       </c>
-      <c r="C37" s="10" t="s">
+      <c r="D37" s="10" t="s">
         <v>138</v>
       </c>
-      <c r="D37" s="10" t="s">
-        <v>157</v>
-      </c>
-      <c r="E37" s="11">
-        <v>46296</v>
-      </c>
-      <c r="F37" s="10" t="s">
-        <v>194</v>
+      <c r="E37" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="F37" s="11">
+        <v>46296</v>
       </c>
       <c r="G37" s="12" t="s">
         <v>308</v>
@@ -2922,25 +3389,33 @@
       <c r="M37" s="3" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="38" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="2" t="s">
+      <c r="N37" s="15" t="s">
+        <v>358</v>
+      </c>
+      <c r="O37" s="19"/>
+      <c r="P37" s="18" t="s">
+        <v>389</v>
+      </c>
+      <c r="Q37" s="18"/>
+    </row>
+    <row r="38" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="B38" s="2" t="s">
         <v>236</v>
       </c>
-      <c r="B38" s="2" t="s">
+      <c r="C38" s="2" t="s">
         <v>291</v>
       </c>
-      <c r="C38" s="10" t="s">
+      <c r="D38" s="10" t="s">
         <v>139</v>
       </c>
-      <c r="D38" s="10" t="s">
-        <v>157</v>
-      </c>
-      <c r="E38" s="11">
-        <v>46296</v>
-      </c>
-      <c r="F38" s="10" t="s">
-        <v>195</v>
+      <c r="E38" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="F38" s="11">
+        <v>46296</v>
       </c>
       <c r="G38" s="12" t="s">
         <v>308</v>
@@ -2959,25 +3434,33 @@
       <c r="M38" s="3" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="39" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="2" t="s">
+      <c r="N38" s="16" t="s">
+        <v>374</v>
+      </c>
+      <c r="O38" s="19"/>
+      <c r="P38" s="18" t="s">
+        <v>386</v>
+      </c>
+      <c r="Q38" s="18"/>
+    </row>
+    <row r="39" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="10" t="s">
+        <v>196</v>
+      </c>
+      <c r="B39" s="2" t="s">
         <v>249</v>
       </c>
-      <c r="B39" s="2" t="s">
+      <c r="C39" s="2" t="s">
         <v>292</v>
       </c>
-      <c r="C39" s="10" t="s">
+      <c r="D39" s="10" t="s">
         <v>140</v>
       </c>
-      <c r="D39" s="10" t="s">
-        <v>157</v>
-      </c>
-      <c r="E39" s="11">
-        <v>46296</v>
-      </c>
-      <c r="F39" s="10" t="s">
-        <v>196</v>
+      <c r="E39" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="F39" s="11">
+        <v>46296</v>
       </c>
       <c r="G39" s="12" t="s">
         <v>308</v>
@@ -2996,25 +3479,33 @@
       <c r="M39" s="3" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="40" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="2" t="s">
+      <c r="N39" s="16" t="s">
+        <v>354</v>
+      </c>
+      <c r="O39" s="19"/>
+      <c r="P39" s="18" t="s">
+        <v>385</v>
+      </c>
+      <c r="Q39" s="18"/>
+    </row>
+    <row r="40" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="10" t="s">
+        <v>197</v>
+      </c>
+      <c r="B40" s="2" t="s">
         <v>250</v>
       </c>
-      <c r="B40" s="2" t="s">
+      <c r="C40" s="2" t="s">
         <v>293</v>
       </c>
-      <c r="C40" s="10" t="s">
+      <c r="D40" s="10" t="s">
         <v>141</v>
       </c>
-      <c r="D40" s="10" t="s">
-        <v>157</v>
-      </c>
-      <c r="E40" s="11">
-        <v>46296</v>
-      </c>
-      <c r="F40" s="10" t="s">
-        <v>197</v>
+      <c r="E40" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="F40" s="11">
+        <v>46296</v>
       </c>
       <c r="G40" s="12" t="s">
         <v>308</v>
@@ -3033,25 +3524,33 @@
       <c r="M40" s="3" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="41" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="2" t="s">
+      <c r="N40" s="16" t="s">
+        <v>354</v>
+      </c>
+      <c r="O40" s="19"/>
+      <c r="P40" s="18" t="s">
+        <v>385</v>
+      </c>
+      <c r="Q40" s="18"/>
+    </row>
+    <row r="41" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="10" t="s">
+        <v>198</v>
+      </c>
+      <c r="B41" s="2" t="s">
         <v>251</v>
       </c>
-      <c r="B41" s="2" t="s">
+      <c r="C41" s="2" t="s">
         <v>294</v>
       </c>
-      <c r="C41" s="10" t="s">
+      <c r="D41" s="10" t="s">
         <v>142</v>
       </c>
-      <c r="D41" s="10" t="s">
-        <v>157</v>
-      </c>
-      <c r="E41" s="11">
-        <v>46296</v>
-      </c>
-      <c r="F41" s="10" t="s">
-        <v>198</v>
+      <c r="E41" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="F41" s="11">
+        <v>46296</v>
       </c>
       <c r="G41" s="12" t="s">
         <v>308</v>
@@ -3070,25 +3569,33 @@
       <c r="M41" s="3" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="42" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="2" t="s">
+      <c r="N41" s="16" t="s">
+        <v>356</v>
+      </c>
+      <c r="O41" s="19"/>
+      <c r="P41" s="18" t="s">
+        <v>385</v>
+      </c>
+      <c r="Q41" s="18"/>
+    </row>
+    <row r="42" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="10" t="s">
+        <v>199</v>
+      </c>
+      <c r="B42" s="2" t="s">
         <v>252</v>
       </c>
-      <c r="B42" s="2" t="s">
+      <c r="C42" s="2" t="s">
         <v>295</v>
       </c>
-      <c r="C42" s="10" t="s">
+      <c r="D42" s="10" t="s">
         <v>143</v>
       </c>
-      <c r="D42" s="10" t="s">
-        <v>157</v>
-      </c>
-      <c r="E42" s="11">
-        <v>46296</v>
-      </c>
-      <c r="F42" s="10" t="s">
-        <v>199</v>
+      <c r="E42" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="F42" s="11">
+        <v>46296</v>
       </c>
       <c r="G42" s="12" t="s">
         <v>308</v>
@@ -3107,25 +3614,33 @@
       <c r="M42" s="3" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="43" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="2" t="s">
+      <c r="N42" s="15" t="s">
+        <v>358</v>
+      </c>
+      <c r="O42" s="19"/>
+      <c r="P42" s="18" t="s">
+        <v>385</v>
+      </c>
+      <c r="Q42" s="18"/>
+    </row>
+    <row r="43" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="10" t="s">
+        <v>200</v>
+      </c>
+      <c r="B43" s="2" t="s">
         <v>253</v>
       </c>
-      <c r="B43" s="2" t="s">
+      <c r="C43" s="2" t="s">
         <v>296</v>
       </c>
-      <c r="C43" s="10" t="s">
+      <c r="D43" s="10" t="s">
         <v>144</v>
       </c>
-      <c r="D43" s="10" t="s">
-        <v>157</v>
-      </c>
-      <c r="E43" s="11">
-        <v>46296</v>
-      </c>
-      <c r="F43" s="10" t="s">
-        <v>200</v>
+      <c r="E43" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="F43" s="11">
+        <v>46296</v>
       </c>
       <c r="G43" s="12" t="s">
         <v>309</v>
@@ -3148,25 +3663,37 @@
       <c r="M43" s="3" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="44" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="2" t="s">
+      <c r="N43" s="16" t="s">
+        <v>369</v>
+      </c>
+      <c r="O43" s="20" t="s">
+        <v>366</v>
+      </c>
+      <c r="P43" s="18" t="s">
+        <v>385</v>
+      </c>
+      <c r="Q43" s="18" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="44" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="10" t="s">
+        <v>201</v>
+      </c>
+      <c r="B44" s="2" t="s">
         <v>232</v>
       </c>
-      <c r="B44" s="2" t="s">
+      <c r="C44" s="2" t="s">
         <v>297</v>
       </c>
-      <c r="C44" s="10" t="s">
+      <c r="D44" s="10" t="s">
         <v>145</v>
       </c>
-      <c r="D44" s="10" t="s">
-        <v>157</v>
-      </c>
-      <c r="E44" s="11">
-        <v>46296</v>
-      </c>
-      <c r="F44" s="10" t="s">
-        <v>201</v>
+      <c r="E44" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="F44" s="11">
+        <v>46296</v>
       </c>
       <c r="G44" s="12" t="s">
         <v>308</v>
@@ -3185,25 +3712,33 @@
       <c r="M44" s="3" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="45" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="2" t="s">
+      <c r="N44" s="16" t="s">
+        <v>369</v>
+      </c>
+      <c r="O44" s="19"/>
+      <c r="P44" s="18" t="s">
+        <v>385</v>
+      </c>
+      <c r="Q44" s="18"/>
+    </row>
+    <row r="45" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="10" t="s">
+        <v>202</v>
+      </c>
+      <c r="B45" s="2" t="s">
         <v>222</v>
       </c>
-      <c r="B45" s="2" t="s">
+      <c r="C45" s="2" t="s">
         <v>298</v>
       </c>
-      <c r="C45" s="10" t="s">
+      <c r="D45" s="10" t="s">
         <v>146</v>
       </c>
-      <c r="D45" s="10" t="s">
-        <v>157</v>
-      </c>
-      <c r="E45" s="11">
-        <v>46296</v>
-      </c>
-      <c r="F45" s="10" t="s">
-        <v>202</v>
+      <c r="E45" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="F45" s="11">
+        <v>46296</v>
       </c>
       <c r="G45" s="12" t="s">
         <v>308</v>
@@ -3222,25 +3757,32 @@
       <c r="M45" s="3" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="46" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="2" t="s">
+      <c r="N45" s="16" t="s">
+        <v>371</v>
+      </c>
+      <c r="P45" s="18" t="s">
+        <v>384</v>
+      </c>
+      <c r="Q45" s="18"/>
+    </row>
+    <row r="46" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="10" t="s">
+        <v>203</v>
+      </c>
+      <c r="B46" s="2" t="s">
         <v>254</v>
       </c>
-      <c r="B46" s="2" t="s">
+      <c r="C46" s="2" t="s">
         <v>299</v>
       </c>
-      <c r="C46" s="10" t="s">
+      <c r="D46" s="10" t="s">
         <v>147</v>
       </c>
-      <c r="D46" s="10" t="s">
-        <v>157</v>
-      </c>
-      <c r="E46" s="11">
-        <v>46296</v>
-      </c>
-      <c r="F46" s="10" t="s">
-        <v>203</v>
+      <c r="E46" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="F46" s="11">
+        <v>46296</v>
       </c>
       <c r="G46" s="12" t="s">
         <v>309</v>
@@ -3263,25 +3805,37 @@
       <c r="M46" s="3" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="47" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="2" t="s">
+      <c r="N46" s="16" t="s">
+        <v>369</v>
+      </c>
+      <c r="O46" s="19" t="s">
+        <v>366</v>
+      </c>
+      <c r="P46" s="18" t="s">
+        <v>385</v>
+      </c>
+      <c r="Q46" s="18" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="47" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="10" t="s">
+        <v>204</v>
+      </c>
+      <c r="B47" s="2" t="s">
         <v>233</v>
       </c>
-      <c r="B47" s="2" t="s">
+      <c r="C47" s="2" t="s">
         <v>300</v>
       </c>
-      <c r="C47" s="10" t="s">
+      <c r="D47" s="10" t="s">
         <v>148</v>
       </c>
-      <c r="D47" s="10" t="s">
-        <v>157</v>
-      </c>
-      <c r="E47" s="11">
-        <v>46296</v>
-      </c>
-      <c r="F47" s="10" t="s">
-        <v>204</v>
+      <c r="E47" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="F47" s="11">
+        <v>46296</v>
       </c>
       <c r="G47" s="12" t="s">
         <v>308</v>
@@ -3300,25 +3854,33 @@
       <c r="M47" s="3" t="s">
         <v>90</v>
       </c>
-    </row>
-    <row r="48" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="2" t="s">
+      <c r="N47" s="16" t="s">
+        <v>369</v>
+      </c>
+      <c r="O47" s="19"/>
+      <c r="P47" s="18" t="s">
+        <v>385</v>
+      </c>
+      <c r="Q47" s="18"/>
+    </row>
+    <row r="48" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="10" t="s">
+        <v>205</v>
+      </c>
+      <c r="B48" s="2" t="s">
         <v>224</v>
       </c>
-      <c r="B48" s="2" t="s">
+      <c r="C48" s="2" t="s">
         <v>301</v>
       </c>
-      <c r="C48" s="10" t="s">
+      <c r="D48" s="10" t="s">
         <v>149</v>
       </c>
-      <c r="D48" s="10" t="s">
-        <v>157</v>
-      </c>
-      <c r="E48" s="11">
-        <v>46296</v>
-      </c>
-      <c r="F48" s="10" t="s">
-        <v>205</v>
+      <c r="E48" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="F48" s="11">
+        <v>46296</v>
       </c>
       <c r="G48" s="12" t="s">
         <v>309</v>
@@ -3337,25 +3899,37 @@
       <c r="M48" s="3" t="s">
         <v>92</v>
       </c>
-    </row>
-    <row r="49" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="2" t="s">
+      <c r="N48" s="15" t="s">
+        <v>371</v>
+      </c>
+      <c r="O48" s="19" t="s">
+        <v>371</v>
+      </c>
+      <c r="P48" s="18" t="s">
+        <v>389</v>
+      </c>
+      <c r="Q48" s="18" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="49" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A49" s="10" t="s">
+        <v>206</v>
+      </c>
+      <c r="B49" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="B49" s="2" t="s">
+      <c r="C49" s="2" t="s">
         <v>302</v>
       </c>
-      <c r="C49" s="10" t="s">
+      <c r="D49" s="10" t="s">
         <v>150</v>
       </c>
-      <c r="D49" s="10" t="s">
-        <v>157</v>
-      </c>
-      <c r="E49" s="11">
-        <v>46296</v>
-      </c>
-      <c r="F49" s="10" t="s">
-        <v>206</v>
+      <c r="E49" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="F49" s="11">
+        <v>46296</v>
       </c>
       <c r="G49" s="12" t="s">
         <v>308</v>
@@ -3374,25 +3948,33 @@
       <c r="M49" s="3" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="50" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="2" t="s">
+      <c r="N49" s="16" t="s">
+        <v>376</v>
+      </c>
+      <c r="O49" s="19"/>
+      <c r="P49" s="18" t="s">
+        <v>384</v>
+      </c>
+      <c r="Q49" s="18"/>
+    </row>
+    <row r="50" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A50" s="10" t="s">
+        <v>207</v>
+      </c>
+      <c r="B50" s="2" t="s">
         <v>235</v>
       </c>
-      <c r="B50" s="2" t="s">
+      <c r="C50" s="2" t="s">
         <v>303</v>
       </c>
-      <c r="C50" s="10" t="s">
+      <c r="D50" s="10" t="s">
         <v>151</v>
       </c>
-      <c r="D50" s="10" t="s">
-        <v>157</v>
-      </c>
-      <c r="E50" s="11">
-        <v>46296</v>
-      </c>
-      <c r="F50" s="10" t="s">
-        <v>207</v>
+      <c r="E50" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="F50" s="11">
+        <v>46296</v>
       </c>
       <c r="G50" s="12" t="s">
         <v>308</v>
@@ -3411,25 +3993,33 @@
       <c r="M50" s="3" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="51" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="2" t="s">
+      <c r="N50" s="16" t="s">
+        <v>381</v>
+      </c>
+      <c r="O50" s="19"/>
+      <c r="P50" s="18" t="s">
+        <v>386</v>
+      </c>
+      <c r="Q50" s="18"/>
+    </row>
+    <row r="51" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A51" s="10" t="s">
+        <v>208</v>
+      </c>
+      <c r="B51" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="B51" s="2" t="s">
+      <c r="C51" s="2" t="s">
         <v>304</v>
       </c>
-      <c r="C51" s="10" t="s">
+      <c r="D51" s="10" t="s">
         <v>152</v>
       </c>
-      <c r="D51" s="10" t="s">
-        <v>157</v>
-      </c>
-      <c r="E51" s="11">
-        <v>46296</v>
-      </c>
-      <c r="F51" s="10" t="s">
-        <v>208</v>
+      <c r="E51" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="F51" s="11">
+        <v>46296</v>
       </c>
       <c r="G51" s="12" t="s">
         <v>308</v>
@@ -3448,25 +4038,33 @@
       <c r="M51" s="3" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="52" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="2" t="s">
+      <c r="N51" s="16" t="s">
+        <v>381</v>
+      </c>
+      <c r="O51" s="19"/>
+      <c r="P51" s="18" t="s">
+        <v>384</v>
+      </c>
+      <c r="Q51" s="18"/>
+    </row>
+    <row r="52" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A52" s="10" t="s">
+        <v>209</v>
+      </c>
+      <c r="B52" s="2" t="s">
         <v>230</v>
       </c>
-      <c r="B52" s="2" t="s">
+      <c r="C52" s="2" t="s">
         <v>305</v>
       </c>
-      <c r="C52" s="10" t="s">
+      <c r="D52" s="10" t="s">
         <v>153</v>
       </c>
-      <c r="D52" s="10" t="s">
-        <v>157</v>
-      </c>
-      <c r="E52" s="11">
-        <v>46296</v>
-      </c>
-      <c r="F52" s="10" t="s">
-        <v>209</v>
+      <c r="E52" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="F52" s="11">
+        <v>46296</v>
       </c>
       <c r="G52" s="12" t="s">
         <v>308</v>
@@ -3485,9 +4083,17 @@
       <c r="M52" s="3" t="s">
         <v>100</v>
       </c>
+      <c r="N52" s="16" t="s">
+        <v>360</v>
+      </c>
+      <c r="O52" s="19"/>
+      <c r="P52" s="18" t="s">
+        <v>385</v>
+      </c>
+      <c r="Q52" s="18"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I52" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="B1:N52" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Tables generating with codes of items
</commit_message>
<xml_diff>
--- a/vars_parsing.xlsx
+++ b/vars_parsing.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\d.sharygin\Desktop\Protocols\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{852CA4D3-4ABC-4340-A224-2F05AE4BEEC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1D7D4AD-452C-44B0-95CC-ACF996AEEA5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="19095" yWindow="0" windowWidth="19410" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="653" uniqueCount="390">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="678" uniqueCount="400">
   <si>
     <t>ЮТКБ.656463.300-001 РЭ</t>
   </si>
@@ -1212,6 +1212,36 @@
   </si>
   <si>
     <t>ЮНИТ-ИЧМ-СУГР-К</t>
+  </si>
+  <si>
+    <t>code_order3</t>
+  </si>
+  <si>
+    <t>ЮНИТ-М519-ДЗШ-Р102-К103-К103-К103-х-х-В101-В101-В101-В101-В101-М1С4.0С00-С01.04</t>
+  </si>
+  <si>
+    <t>ЮНИТ-М519-ДЗШ-Р102-К103-К103-К103-х-х-В101-В101-В101-В101-В101-М1С4.0С00-С01.05</t>
+  </si>
+  <si>
+    <t>ЮНИТ-М519-ДЗШ-Р102-К103-К103-К103-К103-К103-В121-В121-В101-М1С4.0С00-М1С4.0С00-С01.04</t>
+  </si>
+  <si>
+    <t>ЮНИТ-М519-ДЗШ-Р102-К103-К103-К103-К103-К103-В121-В121-В101-М1С4.0С00-М1С4.0С00-С01.05</t>
+  </si>
+  <si>
+    <t>ЮНИТ-М519-ДЗШ-Р102-К103-К103-К103-В121-В121-В121-В121-В101-М1С4.0С00-М1С4.0С00-С01.04</t>
+  </si>
+  <si>
+    <t>ЮНИТ-М519-ДЗШ-Р102-К103-К103-К103-В121-В121-В121-В121-В101-М1С4.0С00-М1С4.0С00-С01.05</t>
+  </si>
+  <si>
+    <t>code_hmi3</t>
+  </si>
+  <si>
+    <t>code_prmprd</t>
+  </si>
+  <si>
+    <t>ПВЗУ-ЕК</t>
   </si>
 </sst>
 </file>
@@ -1675,7 +1705,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q52"/>
+  <dimension ref="A1:T52"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.28515625" style="1" bestFit="1" customWidth="1"/>
@@ -1692,12 +1722,13 @@
     <col min="12" max="12" width="20.5703125" customWidth="1"/>
     <col min="13" max="13" width="23" customWidth="1"/>
     <col min="14" max="14" width="89.42578125" customWidth="1"/>
-    <col min="15" max="15" width="86.140625" customWidth="1"/>
-    <col min="16" max="16" width="26.85546875" customWidth="1"/>
-    <col min="17" max="17" width="23.7109375" customWidth="1"/>
+    <col min="15" max="16" width="86.140625" customWidth="1"/>
+    <col min="17" max="17" width="26.85546875" customWidth="1"/>
+    <col min="18" max="19" width="23.7109375" customWidth="1"/>
+    <col min="20" max="20" width="20.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
         <v>158</v>
       </c>
@@ -1743,14 +1774,23 @@
       <c r="O1" s="17" t="s">
         <v>378</v>
       </c>
-      <c r="P1" s="21" t="s">
+      <c r="P1" s="17" t="s">
+        <v>390</v>
+      </c>
+      <c r="Q1" s="21" t="s">
         <v>383</v>
       </c>
-      <c r="Q1" s="21" t="s">
+      <c r="R1" s="21" t="s">
         <v>387</v>
       </c>
-    </row>
-    <row r="2" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S1" s="21" t="s">
+        <v>397</v>
+      </c>
+      <c r="T1" s="21" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="2" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
         <v>159</v>
       </c>
@@ -1789,13 +1829,24 @@
       <c r="N2" s="16" t="s">
         <v>359</v>
       </c>
-      <c r="O2" s="19"/>
+      <c r="O2" s="18" t="s">
+        <v>391</v>
+      </c>
       <c r="P2" s="18" t="s">
+        <v>392</v>
+      </c>
+      <c r="Q2" s="18" t="s">
         <v>384</v>
       </c>
-      <c r="Q2" s="18"/>
-    </row>
-    <row r="3" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R2" s="18" t="s">
+        <v>384</v>
+      </c>
+      <c r="S2" s="18" t="s">
+        <v>384</v>
+      </c>
+      <c r="T2" s="18"/>
+    </row>
+    <row r="3" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>160</v>
       </c>
@@ -1834,13 +1885,24 @@
       <c r="N3" s="16" t="s">
         <v>362</v>
       </c>
-      <c r="O3" s="19"/>
+      <c r="O3" s="18" t="s">
+        <v>393</v>
+      </c>
       <c r="P3" s="18" t="s">
+        <v>394</v>
+      </c>
+      <c r="Q3" s="18" t="s">
         <v>384</v>
       </c>
-      <c r="Q3" s="18"/>
-    </row>
-    <row r="4" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R3" s="18" t="s">
+        <v>384</v>
+      </c>
+      <c r="S3" s="18" t="s">
+        <v>384</v>
+      </c>
+      <c r="T3" s="18"/>
+    </row>
+    <row r="4" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>161</v>
       </c>
@@ -1879,13 +1941,24 @@
       <c r="N4" s="16" t="s">
         <v>359</v>
       </c>
-      <c r="O4" s="19"/>
+      <c r="O4" s="18" t="s">
+        <v>391</v>
+      </c>
       <c r="P4" s="18" t="s">
+        <v>392</v>
+      </c>
+      <c r="Q4" s="18" t="s">
         <v>384</v>
       </c>
-      <c r="Q4" s="18"/>
-    </row>
-    <row r="5" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R4" s="18" t="s">
+        <v>384</v>
+      </c>
+      <c r="S4" s="18" t="s">
+        <v>384</v>
+      </c>
+      <c r="T4" s="18"/>
+    </row>
+    <row r="5" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>162</v>
       </c>
@@ -1924,13 +1997,24 @@
       <c r="N5" s="16" t="s">
         <v>363</v>
       </c>
-      <c r="O5" s="19"/>
+      <c r="O5" s="18" t="s">
+        <v>395</v>
+      </c>
       <c r="P5" s="18" t="s">
+        <v>396</v>
+      </c>
+      <c r="Q5" s="18" t="s">
         <v>384</v>
       </c>
-      <c r="Q5" s="18"/>
-    </row>
-    <row r="6" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R5" s="18" t="s">
+        <v>384</v>
+      </c>
+      <c r="S5" s="18" t="s">
+        <v>384</v>
+      </c>
+      <c r="T5" s="18"/>
+    </row>
+    <row r="6" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>163</v>
       </c>
@@ -1972,14 +2056,17 @@
       <c r="O6" s="19" t="s">
         <v>365</v>
       </c>
-      <c r="P6" s="18" t="s">
-        <v>384</v>
-      </c>
+      <c r="P6" s="19"/>
       <c r="Q6" s="18" t="s">
         <v>384</v>
       </c>
-    </row>
-    <row r="7" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R6" s="18" t="s">
+        <v>384</v>
+      </c>
+      <c r="S6" s="18"/>
+      <c r="T6" s="18"/>
+    </row>
+    <row r="7" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
         <v>164</v>
       </c>
@@ -2019,12 +2106,15 @@
         <v>365</v>
       </c>
       <c r="O7" s="19"/>
-      <c r="P7" s="18" t="s">
+      <c r="P7" s="19"/>
+      <c r="Q7" s="18" t="s">
         <v>384</v>
       </c>
-      <c r="Q7" s="18"/>
-    </row>
-    <row r="8" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R7" s="18"/>
+      <c r="S7" s="18"/>
+      <c r="T7" s="18"/>
+    </row>
+    <row r="8" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>165</v>
       </c>
@@ -2064,12 +2154,15 @@
         <v>357</v>
       </c>
       <c r="O8" s="19"/>
-      <c r="P8" s="18" t="s">
+      <c r="P8" s="19"/>
+      <c r="Q8" s="18" t="s">
         <v>384</v>
       </c>
-      <c r="Q8" s="18"/>
-    </row>
-    <row r="9" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R8" s="18"/>
+      <c r="S8" s="18"/>
+      <c r="T8" s="18"/>
+    </row>
+    <row r="9" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
         <v>166</v>
       </c>
@@ -2109,12 +2202,15 @@
         <v>373</v>
       </c>
       <c r="O9" s="19"/>
-      <c r="P9" s="18" t="s">
+      <c r="P9" s="19"/>
+      <c r="Q9" s="18" t="s">
         <v>384</v>
       </c>
-      <c r="Q9" s="18"/>
-    </row>
-    <row r="10" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R9" s="18"/>
+      <c r="S9" s="18"/>
+      <c r="T9" s="18"/>
+    </row>
+    <row r="10" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="10" t="s">
         <v>167</v>
       </c>
@@ -2154,12 +2250,15 @@
         <v>357</v>
       </c>
       <c r="O10" s="19"/>
-      <c r="P10" s="18" t="s">
+      <c r="P10" s="19"/>
+      <c r="Q10" s="18" t="s">
         <v>384</v>
       </c>
-      <c r="Q10" s="18"/>
-    </row>
-    <row r="11" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R10" s="18"/>
+      <c r="S10" s="18"/>
+      <c r="T10" s="18"/>
+    </row>
+    <row r="11" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="10" t="s">
         <v>168</v>
       </c>
@@ -2199,12 +2298,15 @@
         <v>379</v>
       </c>
       <c r="O11" s="19"/>
-      <c r="P11" s="18" t="s">
+      <c r="P11" s="19"/>
+      <c r="Q11" s="18" t="s">
         <v>384</v>
       </c>
-      <c r="Q11" s="18"/>
-    </row>
-    <row r="12" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R11" s="18"/>
+      <c r="S11" s="18"/>
+      <c r="T11" s="18"/>
+    </row>
+    <row r="12" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="10" t="s">
         <v>169</v>
       </c>
@@ -2244,12 +2346,17 @@
         <v>353</v>
       </c>
       <c r="O12" s="19"/>
-      <c r="P12" s="18" t="s">
+      <c r="P12" s="19"/>
+      <c r="Q12" s="18" t="s">
         <v>384</v>
       </c>
-      <c r="Q12" s="18"/>
-    </row>
-    <row r="13" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R12" s="18"/>
+      <c r="S12" s="18"/>
+      <c r="T12" s="18" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="13" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="10" t="s">
         <v>170</v>
       </c>
@@ -2289,12 +2396,17 @@
         <v>353</v>
       </c>
       <c r="O13" s="19"/>
-      <c r="P13" s="18" t="s">
+      <c r="P13" s="19"/>
+      <c r="Q13" s="18" t="s">
         <v>384</v>
       </c>
-      <c r="Q13" s="18"/>
-    </row>
-    <row r="14" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R13" s="18"/>
+      <c r="S13" s="18"/>
+      <c r="T13" s="18" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="14" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="10" t="s">
         <v>171</v>
       </c>
@@ -2334,12 +2446,17 @@
         <v>353</v>
       </c>
       <c r="O14" s="19"/>
-      <c r="P14" s="18" t="s">
+      <c r="P14" s="19"/>
+      <c r="Q14" s="18" t="s">
         <v>384</v>
       </c>
-      <c r="Q14" s="18"/>
-    </row>
-    <row r="15" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R14" s="18"/>
+      <c r="S14" s="18"/>
+      <c r="T14" s="18" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="15" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="10" t="s">
         <v>172</v>
       </c>
@@ -2379,12 +2496,17 @@
         <v>353</v>
       </c>
       <c r="O15" s="19"/>
-      <c r="P15" s="18" t="s">
+      <c r="P15" s="19"/>
+      <c r="Q15" s="18" t="s">
         <v>384</v>
       </c>
-      <c r="Q15" s="18"/>
-    </row>
-    <row r="16" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R15" s="18"/>
+      <c r="S15" s="18"/>
+      <c r="T15" s="18" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="16" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="10" t="s">
         <v>173</v>
       </c>
@@ -2424,12 +2546,15 @@
         <v>355</v>
       </c>
       <c r="O16" s="19"/>
-      <c r="P16" s="18" t="s">
+      <c r="P16" s="19"/>
+      <c r="Q16" s="18" t="s">
         <v>384</v>
       </c>
-      <c r="Q16" s="18"/>
-    </row>
-    <row r="17" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R16" s="18"/>
+      <c r="S16" s="18"/>
+      <c r="T16" s="18"/>
+    </row>
+    <row r="17" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="10" t="s">
         <v>174</v>
       </c>
@@ -2469,12 +2594,15 @@
         <v>355</v>
       </c>
       <c r="O17" s="19"/>
-      <c r="P17" s="18" t="s">
+      <c r="P17" s="19"/>
+      <c r="Q17" s="18" t="s">
         <v>384</v>
       </c>
-      <c r="Q17" s="18"/>
-    </row>
-    <row r="18" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R17" s="18"/>
+      <c r="S17" s="18"/>
+      <c r="T17" s="18"/>
+    </row>
+    <row r="18" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="10" t="s">
         <v>175</v>
       </c>
@@ -2514,12 +2642,15 @@
         <v>357</v>
       </c>
       <c r="O18" s="19"/>
-      <c r="P18" s="18" t="s">
+      <c r="P18" s="19"/>
+      <c r="Q18" s="18" t="s">
         <v>384</v>
       </c>
-      <c r="Q18" s="18"/>
-    </row>
-    <row r="19" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R18" s="18"/>
+      <c r="S18" s="18"/>
+      <c r="T18" s="18"/>
+    </row>
+    <row r="19" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="10" t="s">
         <v>176</v>
       </c>
@@ -2559,12 +2690,15 @@
         <v>357</v>
       </c>
       <c r="O19" s="19"/>
-      <c r="P19" s="18" t="s">
+      <c r="P19" s="19"/>
+      <c r="Q19" s="18" t="s">
         <v>384</v>
       </c>
-      <c r="Q19" s="18"/>
-    </row>
-    <row r="20" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R19" s="18"/>
+      <c r="S19" s="18"/>
+      <c r="T19" s="18"/>
+    </row>
+    <row r="20" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="10" t="s">
         <v>177</v>
       </c>
@@ -2604,12 +2738,15 @@
         <v>357</v>
       </c>
       <c r="O20" s="19"/>
-      <c r="P20" s="18" t="s">
+      <c r="P20" s="19"/>
+      <c r="Q20" s="18" t="s">
         <v>384</v>
       </c>
-      <c r="Q20" s="18"/>
-    </row>
-    <row r="21" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R20" s="18"/>
+      <c r="S20" s="18"/>
+      <c r="T20" s="18"/>
+    </row>
+    <row r="21" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="10" t="s">
         <v>178</v>
       </c>
@@ -2655,14 +2792,17 @@
       <c r="O21" s="20" t="s">
         <v>365</v>
       </c>
-      <c r="P21" s="18" t="s">
+      <c r="P21" s="20"/>
+      <c r="Q21" s="18" t="s">
         <v>386</v>
       </c>
-      <c r="Q21" s="18" t="s">
+      <c r="R21" s="18" t="s">
         <v>384</v>
       </c>
-    </row>
-    <row r="22" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S21" s="18"/>
+      <c r="T21" s="18"/>
+    </row>
+    <row r="22" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="10" t="s">
         <v>179</v>
       </c>
@@ -2702,12 +2842,15 @@
         <v>368</v>
       </c>
       <c r="O22" s="19"/>
-      <c r="P22" s="18" t="s">
+      <c r="P22" s="19"/>
+      <c r="Q22" s="18" t="s">
         <v>385</v>
       </c>
-      <c r="Q22" s="18"/>
-    </row>
-    <row r="23" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R22" s="18"/>
+      <c r="S22" s="18"/>
+      <c r="T22" s="18"/>
+    </row>
+    <row r="23" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="10" t="s">
         <v>180</v>
       </c>
@@ -2747,12 +2890,15 @@
         <v>370</v>
       </c>
       <c r="O23" s="19"/>
-      <c r="P23" s="18" t="s">
+      <c r="P23" s="19"/>
+      <c r="Q23" s="18" t="s">
         <v>384</v>
       </c>
-      <c r="Q23" s="18"/>
-    </row>
-    <row r="24" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R23" s="18"/>
+      <c r="S23" s="18"/>
+      <c r="T23" s="18"/>
+    </row>
+    <row r="24" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="10" t="s">
         <v>181</v>
       </c>
@@ -2798,14 +2944,17 @@
       <c r="O24" s="19" t="s">
         <v>365</v>
       </c>
-      <c r="P24" s="18" t="s">
+      <c r="P24" s="19"/>
+      <c r="Q24" s="18" t="s">
         <v>386</v>
       </c>
-      <c r="Q24" s="18" t="s">
+      <c r="R24" s="18" t="s">
         <v>384</v>
       </c>
-    </row>
-    <row r="25" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S24" s="18"/>
+      <c r="T24" s="18"/>
+    </row>
+    <row r="25" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="10" t="s">
         <v>182</v>
       </c>
@@ -2845,12 +2994,15 @@
         <v>368</v>
       </c>
       <c r="O25" s="19"/>
-      <c r="P25" s="18" t="s">
+      <c r="P25" s="19"/>
+      <c r="Q25" s="18" t="s">
         <v>386</v>
       </c>
-      <c r="Q25" s="18"/>
-    </row>
-    <row r="26" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R25" s="18"/>
+      <c r="S25" s="18"/>
+      <c r="T25" s="18"/>
+    </row>
+    <row r="26" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="10" t="s">
         <v>183</v>
       </c>
@@ -2890,12 +3042,15 @@
         <v>372</v>
       </c>
       <c r="O26" s="19"/>
-      <c r="P26" s="18" t="s">
+      <c r="P26" s="19"/>
+      <c r="Q26" s="18" t="s">
         <v>384</v>
       </c>
-      <c r="Q26" s="18"/>
-    </row>
-    <row r="27" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R26" s="18"/>
+      <c r="S26" s="18"/>
+      <c r="T26" s="18"/>
+    </row>
+    <row r="27" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="10" t="s">
         <v>184</v>
       </c>
@@ -2935,12 +3090,15 @@
         <v>375</v>
       </c>
       <c r="O27" s="19"/>
-      <c r="P27" s="18" t="s">
+      <c r="P27" s="19"/>
+      <c r="Q27" s="18" t="s">
         <v>384</v>
       </c>
-      <c r="Q27" s="18"/>
-    </row>
-    <row r="28" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R27" s="18"/>
+      <c r="S27" s="18"/>
+      <c r="T27" s="18"/>
+    </row>
+    <row r="28" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="10" t="s">
         <v>185</v>
       </c>
@@ -2982,14 +3140,17 @@
       <c r="O28" s="19" t="s">
         <v>377</v>
       </c>
-      <c r="P28" s="18" t="s">
-        <v>384</v>
-      </c>
+      <c r="P28" s="19"/>
       <c r="Q28" s="18" t="s">
         <v>384</v>
       </c>
-    </row>
-    <row r="29" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R28" s="18" t="s">
+        <v>384</v>
+      </c>
+      <c r="S28" s="18"/>
+      <c r="T28" s="18"/>
+    </row>
+    <row r="29" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="10" t="s">
         <v>186</v>
       </c>
@@ -3029,12 +3190,15 @@
         <v>380</v>
       </c>
       <c r="O29" s="19"/>
-      <c r="P29" s="18" t="s">
+      <c r="P29" s="19"/>
+      <c r="Q29" s="18" t="s">
         <v>386</v>
       </c>
-      <c r="Q29" s="18"/>
-    </row>
-    <row r="30" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R29" s="18"/>
+      <c r="S29" s="18"/>
+      <c r="T29" s="18"/>
+    </row>
+    <row r="30" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="10" t="s">
         <v>187</v>
       </c>
@@ -3074,12 +3238,15 @@
         <v>380</v>
       </c>
       <c r="O30" s="19"/>
-      <c r="P30" s="18" t="s">
+      <c r="P30" s="19"/>
+      <c r="Q30" s="18" t="s">
         <v>384</v>
       </c>
-      <c r="Q30" s="18"/>
-    </row>
-    <row r="31" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R30" s="18"/>
+      <c r="S30" s="18"/>
+      <c r="T30" s="18"/>
+    </row>
+    <row r="31" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="10" t="s">
         <v>188</v>
       </c>
@@ -3119,12 +3286,15 @@
         <v>382</v>
       </c>
       <c r="O31" s="19"/>
-      <c r="P31" s="18" t="s">
+      <c r="P31" s="19"/>
+      <c r="Q31" s="18" t="s">
         <v>384</v>
       </c>
-      <c r="Q31" s="18"/>
-    </row>
-    <row r="32" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R31" s="18"/>
+      <c r="S31" s="18"/>
+      <c r="T31" s="18"/>
+    </row>
+    <row r="32" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="10" t="s">
         <v>189</v>
       </c>
@@ -3164,12 +3334,15 @@
         <v>359</v>
       </c>
       <c r="O32" s="19"/>
-      <c r="P32" s="18" t="s">
+      <c r="P32" s="19"/>
+      <c r="Q32" s="18" t="s">
         <v>384</v>
       </c>
-      <c r="Q32" s="18"/>
-    </row>
-    <row r="33" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R32" s="18"/>
+      <c r="S32" s="18"/>
+      <c r="T32" s="18"/>
+    </row>
+    <row r="33" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="10" t="s">
         <v>190</v>
       </c>
@@ -3209,12 +3382,15 @@
         <v>361</v>
       </c>
       <c r="O33" s="19"/>
-      <c r="P33" s="18" t="s">
+      <c r="P33" s="19"/>
+      <c r="Q33" s="18" t="s">
         <v>385</v>
       </c>
-      <c r="Q33" s="18"/>
-    </row>
-    <row r="34" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R33" s="18"/>
+      <c r="S33" s="18"/>
+      <c r="T33" s="18"/>
+    </row>
+    <row r="34" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="10" t="s">
         <v>191</v>
       </c>
@@ -3254,12 +3430,15 @@
         <v>364</v>
       </c>
       <c r="O34" s="19"/>
-      <c r="P34" s="18" t="s">
+      <c r="P34" s="19"/>
+      <c r="Q34" s="18" t="s">
         <v>388</v>
       </c>
-      <c r="Q34" s="18"/>
-    </row>
-    <row r="35" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R34" s="18"/>
+      <c r="S34" s="18"/>
+      <c r="T34" s="18"/>
+    </row>
+    <row r="35" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="10" t="s">
         <v>192</v>
       </c>
@@ -3301,14 +3480,17 @@
       <c r="O35" s="19" t="s">
         <v>367</v>
       </c>
-      <c r="P35" s="18" t="s">
-        <v>385</v>
-      </c>
+      <c r="P35" s="19"/>
       <c r="Q35" s="18" t="s">
         <v>385</v>
       </c>
-    </row>
-    <row r="36" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R35" s="18" t="s">
+        <v>385</v>
+      </c>
+      <c r="S35" s="18"/>
+      <c r="T35" s="18"/>
+    </row>
+    <row r="36" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="10" t="s">
         <v>193</v>
       </c>
@@ -3348,12 +3530,15 @@
         <v>367</v>
       </c>
       <c r="O36" s="19"/>
-      <c r="P36" s="18" t="s">
+      <c r="P36" s="19"/>
+      <c r="Q36" s="18" t="s">
         <v>385</v>
       </c>
-      <c r="Q36" s="18"/>
-    </row>
-    <row r="37" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R36" s="18"/>
+      <c r="S36" s="18"/>
+      <c r="T36" s="18"/>
+    </row>
+    <row r="37" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="10" t="s">
         <v>194</v>
       </c>
@@ -3393,12 +3578,15 @@
         <v>358</v>
       </c>
       <c r="O37" s="19"/>
-      <c r="P37" s="18" t="s">
+      <c r="P37" s="19"/>
+      <c r="Q37" s="18" t="s">
         <v>389</v>
       </c>
-      <c r="Q37" s="18"/>
-    </row>
-    <row r="38" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R37" s="18"/>
+      <c r="S37" s="18"/>
+      <c r="T37" s="18"/>
+    </row>
+    <row r="38" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="10" t="s">
         <v>195</v>
       </c>
@@ -3438,12 +3626,15 @@
         <v>374</v>
       </c>
       <c r="O38" s="19"/>
-      <c r="P38" s="18" t="s">
+      <c r="P38" s="19"/>
+      <c r="Q38" s="18" t="s">
         <v>386</v>
       </c>
-      <c r="Q38" s="18"/>
-    </row>
-    <row r="39" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R38" s="18"/>
+      <c r="S38" s="18"/>
+      <c r="T38" s="18"/>
+    </row>
+    <row r="39" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="10" t="s">
         <v>196</v>
       </c>
@@ -3483,12 +3674,17 @@
         <v>354</v>
       </c>
       <c r="O39" s="19"/>
-      <c r="P39" s="18" t="s">
+      <c r="P39" s="19"/>
+      <c r="Q39" s="18" t="s">
         <v>385</v>
       </c>
-      <c r="Q39" s="18"/>
-    </row>
-    <row r="40" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R39" s="18"/>
+      <c r="S39" s="18"/>
+      <c r="T39" s="18" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="40" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="10" t="s">
         <v>197</v>
       </c>
@@ -3528,12 +3724,17 @@
         <v>354</v>
       </c>
       <c r="O40" s="19"/>
-      <c r="P40" s="18" t="s">
+      <c r="P40" s="19"/>
+      <c r="Q40" s="18" t="s">
         <v>385</v>
       </c>
-      <c r="Q40" s="18"/>
-    </row>
-    <row r="41" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R40" s="18"/>
+      <c r="S40" s="18"/>
+      <c r="T40" s="18" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="41" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="10" t="s">
         <v>198</v>
       </c>
@@ -3573,12 +3774,15 @@
         <v>356</v>
       </c>
       <c r="O41" s="19"/>
-      <c r="P41" s="18" t="s">
+      <c r="P41" s="19"/>
+      <c r="Q41" s="18" t="s">
         <v>385</v>
       </c>
-      <c r="Q41" s="18"/>
-    </row>
-    <row r="42" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R41" s="18"/>
+      <c r="S41" s="18"/>
+      <c r="T41" s="18"/>
+    </row>
+    <row r="42" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="10" t="s">
         <v>199</v>
       </c>
@@ -3618,12 +3822,15 @@
         <v>358</v>
       </c>
       <c r="O42" s="19"/>
-      <c r="P42" s="18" t="s">
+      <c r="P42" s="19"/>
+      <c r="Q42" s="18" t="s">
         <v>385</v>
       </c>
-      <c r="Q42" s="18"/>
-    </row>
-    <row r="43" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R42" s="18"/>
+      <c r="S42" s="18"/>
+      <c r="T42" s="18"/>
+    </row>
+    <row r="43" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="10" t="s">
         <v>200</v>
       </c>
@@ -3669,14 +3876,17 @@
       <c r="O43" s="20" t="s">
         <v>366</v>
       </c>
-      <c r="P43" s="18" t="s">
+      <c r="P43" s="20"/>
+      <c r="Q43" s="18" t="s">
         <v>385</v>
       </c>
-      <c r="Q43" s="18" t="s">
+      <c r="R43" s="18" t="s">
         <v>384</v>
       </c>
-    </row>
-    <row r="44" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S43" s="18"/>
+      <c r="T43" s="18"/>
+    </row>
+    <row r="44" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="10" t="s">
         <v>201</v>
       </c>
@@ -3716,12 +3926,15 @@
         <v>369</v>
       </c>
       <c r="O44" s="19"/>
-      <c r="P44" s="18" t="s">
+      <c r="P44" s="19"/>
+      <c r="Q44" s="18" t="s">
         <v>385</v>
       </c>
-      <c r="Q44" s="18"/>
-    </row>
-    <row r="45" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R44" s="18"/>
+      <c r="S44" s="18"/>
+      <c r="T44" s="18"/>
+    </row>
+    <row r="45" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="10" t="s">
         <v>202</v>
       </c>
@@ -3760,12 +3973,15 @@
       <c r="N45" s="16" t="s">
         <v>371</v>
       </c>
-      <c r="P45" s="18" t="s">
+      <c r="O45" s="18"/>
+      <c r="Q45" s="18" t="s">
         <v>384</v>
       </c>
-      <c r="Q45" s="18"/>
-    </row>
-    <row r="46" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R45" s="18"/>
+      <c r="S45" s="18"/>
+      <c r="T45" s="18"/>
+    </row>
+    <row r="46" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="10" t="s">
         <v>203</v>
       </c>
@@ -3811,14 +4027,17 @@
       <c r="O46" s="19" t="s">
         <v>366</v>
       </c>
-      <c r="P46" s="18" t="s">
+      <c r="P46" s="19"/>
+      <c r="Q46" s="18" t="s">
         <v>385</v>
       </c>
-      <c r="Q46" s="18" t="s">
+      <c r="R46" s="18" t="s">
         <v>384</v>
       </c>
-    </row>
-    <row r="47" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S46" s="18"/>
+      <c r="T46" s="18"/>
+    </row>
+    <row r="47" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="10" t="s">
         <v>204</v>
       </c>
@@ -3858,12 +4077,15 @@
         <v>369</v>
       </c>
       <c r="O47" s="19"/>
-      <c r="P47" s="18" t="s">
+      <c r="P47" s="19"/>
+      <c r="Q47" s="18" t="s">
         <v>385</v>
       </c>
-      <c r="Q47" s="18"/>
-    </row>
-    <row r="48" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R47" s="18"/>
+      <c r="S47" s="18"/>
+      <c r="T47" s="18"/>
+    </row>
+    <row r="48" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="10" t="s">
         <v>205</v>
       </c>
@@ -3905,14 +4127,17 @@
       <c r="O48" s="19" t="s">
         <v>371</v>
       </c>
-      <c r="P48" s="18" t="s">
-        <v>389</v>
-      </c>
+      <c r="P48" s="19"/>
       <c r="Q48" s="18" t="s">
         <v>389</v>
       </c>
-    </row>
-    <row r="49" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R48" s="18" t="s">
+        <v>389</v>
+      </c>
+      <c r="S48" s="18"/>
+      <c r="T48" s="18"/>
+    </row>
+    <row r="49" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="10" t="s">
         <v>206</v>
       </c>
@@ -3952,12 +4177,15 @@
         <v>376</v>
       </c>
       <c r="O49" s="19"/>
-      <c r="P49" s="18" t="s">
+      <c r="P49" s="19"/>
+      <c r="Q49" s="18" t="s">
         <v>384</v>
       </c>
-      <c r="Q49" s="18"/>
-    </row>
-    <row r="50" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R49" s="18"/>
+      <c r="S49" s="18"/>
+      <c r="T49" s="18"/>
+    </row>
+    <row r="50" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="10" t="s">
         <v>207</v>
       </c>
@@ -3997,12 +4225,15 @@
         <v>381</v>
       </c>
       <c r="O50" s="19"/>
-      <c r="P50" s="18" t="s">
+      <c r="P50" s="19"/>
+      <c r="Q50" s="18" t="s">
         <v>386</v>
       </c>
-      <c r="Q50" s="18"/>
-    </row>
-    <row r="51" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R50" s="18"/>
+      <c r="S50" s="18"/>
+      <c r="T50" s="18"/>
+    </row>
+    <row r="51" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="10" t="s">
         <v>208</v>
       </c>
@@ -4042,12 +4273,15 @@
         <v>381</v>
       </c>
       <c r="O51" s="19"/>
-      <c r="P51" s="18" t="s">
+      <c r="P51" s="19"/>
+      <c r="Q51" s="18" t="s">
         <v>384</v>
       </c>
-      <c r="Q51" s="18"/>
-    </row>
-    <row r="52" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R51" s="18"/>
+      <c r="S51" s="18"/>
+      <c r="T51" s="18"/>
+    </row>
+    <row r="52" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="10" t="s">
         <v>209</v>
       </c>
@@ -4087,10 +4321,13 @@
         <v>360</v>
       </c>
       <c r="O52" s="19"/>
-      <c r="P52" s="18" t="s">
+      <c r="P52" s="19"/>
+      <c r="Q52" s="18" t="s">
         <v>385</v>
       </c>
-      <c r="Q52" s="18"/>
+      <c r="R52" s="18"/>
+      <c r="S52" s="18"/>
+      <c r="T52" s="18"/>
     </row>
   </sheetData>
   <autoFilter ref="B1:N52" xr:uid="{00000000-0001-0000-0000-000000000000}"/>

</xml_diff>